<commit_message>
1. convert data from json to hashmap and use it in body 2. convert data from excel to arraylist and array list to  hashmap and use it in body
</commit_message>
<xml_diff>
--- a/src/main/resources/ReadExcel.xlsx
+++ b/src/main/resources/ReadExcel.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\AKSHAY\new-eclipse-workspace\APIRestAssured2\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C69B6C93-38B0-474D-922E-0D9FFBDF3F54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DBC1B473-34AA-47A6-8B1B-290D14873A58}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-23148" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{6443DC5A-AF05-4B6B-BC56-29A424E9BAAC}"/>
+    <workbookView xWindow="-23148" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{6443DC5A-AF05-4B6B-BC56-29A424E9BAAC}"/>
   </bookViews>
   <sheets>
     <sheet name="testData" sheetId="1" r:id="rId1"/>
-    <sheet name="sample" sheetId="2" r:id="rId2"/>
-    <sheet name="demo" sheetId="3" r:id="rId3"/>
+    <sheet name="RestAssured" sheetId="4" r:id="rId2"/>
+    <sheet name="sample" sheetId="2" r:id="rId3"/>
+    <sheet name="demo" sheetId="3" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="31">
   <si>
     <t>Testcases</t>
   </si>
@@ -99,6 +100,36 @@
   </si>
   <si>
     <t>d</t>
+  </si>
+  <si>
+    <t>RestAddBook</t>
+  </si>
+  <si>
+    <t>Data4</t>
+  </si>
+  <si>
+    <t>Akshay</t>
+  </si>
+  <si>
+    <t>RestAssured</t>
+  </si>
+  <si>
+    <t>bcd</t>
+  </si>
+  <si>
+    <t>name</t>
+  </si>
+  <si>
+    <t>isbn</t>
+  </si>
+  <si>
+    <t>aisle</t>
+  </si>
+  <si>
+    <t>author</t>
+  </si>
+  <si>
+    <t>Testcase</t>
   </si>
 </sst>
 </file>
@@ -128,7 +159,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -151,13 +182,26 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -472,7 +516,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C3EA9D33-94E0-4AA6-A1B8-239DDD2C398C}">
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="11.7109375" bestFit="1" customWidth="1"/>
@@ -480,7 +524,7 @@
     <col min="4" max="4" width="12.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -493,8 +537,11 @@
       <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E1" s="2" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>4</v>
       </c>
@@ -508,7 +555,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>5</v>
       </c>
@@ -522,7 +569,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
         <v>6</v>
       </c>
@@ -536,7 +583,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
         <v>7</v>
       </c>
@@ -548,6 +595,23 @@
       </c>
       <c r="D5" s="1" t="s">
         <v>19</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A6" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="D6" s="2">
+        <v>3126</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>23</v>
       </c>
     </row>
   </sheetData>
@@ -557,6 +621,54 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{212EC1E6-ADD4-4D2E-8619-88686338A27B}">
+  <dimension ref="A1:E2"/>
+  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.85546875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A2" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="D2" s="3">
+        <v>3127</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>23</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{039E0EEF-68F7-4A29-B740-610EAF60A04D}">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
@@ -565,7 +677,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{85E91E2F-FCEF-4570-AE9C-E2FE9FCA06AB}">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>

</xml_diff>